<commit_message>
Publish checkmi r44: two upload templates, dynamic years and account details
</commit_message>
<xml_diff>
--- a/public/checkmi/templates/经营测算_标准底表.xlsx
+++ b/public/checkmi/templates/经营测算_标准底表.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="R63d92dc3348a4280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据填写" sheetId="2" r:id="R22143803667c4c34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例" sheetId="3" r:id="R031a43616a404080"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="R49e1aa16fb564a34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据填写" sheetId="2" r:id="R26492b1541ef4fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例" sheetId="3" r:id="Rc466b528802446dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -403,7 +403,7 @@
       <x:c r="B6" s="11"/>
       <x:c r="C6" s="11"/>
       <x:c r="D6" s="12" t="str">
-        <x:v>保存 .xlsx 后回到看板「接入数据」，查看预览并应用。空模板须填入真实数据后才能导入。</x:v>
+        <x:v>保存.xlsx后在看板选择“上传标准底表”，查看预览并应用。空模板须先填写数据。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
@@ -423,7 +423,7 @@
       <x:c r="B8" s="11"/>
       <x:c r="C8" s="11"/>
       <x:c r="D8" s="12" t="str">
-        <x:v>本模板提供经营必需的合计科目，不含子科目拆分和现金流计划。完整损益子科目请使用原结构 BC 工作簿。</x:v>
+        <x:v>本模板按车型年度填写合计科目；需保留完整子科目时，请下载“损益表模板”并选择“上传损益表”。两者均不含投资现金流。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -513,7 +513,7 @@
         <x:v>SOP</x:v>
       </x:c>
       <x:c r="D15" s="19" t="str">
-        <x:v>SOP、SOP+1 至 SOP+4，或 2026 等年份；同一文件不要混用</x:v>
+        <x:v>SOP、SOP+n（如SOP+8），或2026等年份；同一文件不要混用。增删记录即可增删年度。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="39" customHeight="1">

</xml_diff>